<commit_message>
feat: business_context.txt — magazyny i handlowcy + integracja z nlp_pipeline (backlog id=3)
</commit_message>
<xml_diff>
--- a/solutions/bi/MagElem/MagElem_plan.xlsx
+++ b/solutions/bi/MagElem/MagElem_plan.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kod towaru</t>
+          <t>Kod towaru (aktualny)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -815,13 +815,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Duplikat aliasu — Kod_Towaru pochodzi z MaE_TwrKod (row 9); JOIN TwrKarty tylko dla Nazwa_Towaru</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>MaE_TwrKod dostępne bezpośrednio ale JOIN daje aktualny kod</t>
+          <t>Poprawka iteracja 2 — usunięcie duplikatu (Analityk msg 141)</t>
         </is>
       </c>
     </row>

</xml_diff>